<commit_message>
Leave payment due date (支払期限) blank on both invoices
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xo4ocWdfAKqvEfGtNoNEwm
</commit_message>
<xml_diff>
--- a/invoice/invoice_soren_2026-07.xlsx
+++ b/invoice/invoice_soren_2026-07.xlsx
@@ -661,11 +661,7 @@
           <t>支払期限</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>2026/08/31</t>
-        </is>
-      </c>
+      <c r="E7" s="6" t="inlineStr"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="9" t="inlineStr">

</xml_diff>